<commit_message>
Proposal: editorial pass, consistent review period and renewal reminders, final screens
Cover letter as a business letter; one-page executive summary; cross-
references instead of repetition; consistent terminology, spelling and
money format; journey references computed from the chapter; ten-business-
day document review throughout; renewal reminders aligned with the
45-day window; pricing workbook and bill of materials rebuilt.
</commit_message>
<xml_diff>
--- a/docs/proposal/IIFT-Bill-of-Materials-iorta-TechNXT.xlsx
+++ b/docs/proposal/IIFT-Bill-of-Materials-iorta-TechNXT.xlsx
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Secrets store and customer-managed encryption keys</t>
+          <t>Secrets store and encryption keys held in IIFT's account</t>
         </is>
       </c>
       <c r="E13" s="8" t="n">
@@ -3611,7 +3611,7 @@
     <row r="48" ht="13" customHeight="1">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>•  Direct runtime dependencies: 27 in the API (apps/api/package.json) and 8 in the web application (apps/web/package.json).</t>
+          <t>•  Direct runtime dependencies: 28 in the API (apps/api/package.json) and 8 in the web application (apps/web/package.json).</t>
         </is>
       </c>
     </row>

</xml_diff>